<commit_message>
feat(probabilistic-programming): ship T5 topic 3 — PyMC/NumPyro/Stan dispatch + eight-schools workflow
Closes the Bayesian-machinery arc opened by variational-inference and
gaussian-processes by lifting the modeling step into an executable DSL:
the user writes only the generative model, and the PPL manufactures the
joint log-density, gradients, and constrained-to-unconstrained transforms.
Walks the full Bayesian workflow on Rubin's eight-schools dataset
including the centered-vs-non-centered reparameterization that turns
several-hundred divergences into zero.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R44"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3707,6 +3707,80 @@
       <c r="R44" t="inlineStr">
         <is>
           <t>Overview, 1. From parametric Bayes to function-space priors, 2. Gaussian processes as priors over functions, 3. Conjugate GP regression, 4. Kernel design and the inductive bias, 5. Learning hyperparameters from the marginal likelihood, 6. Scaling, neighbors, and limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>bayesian-ml</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Probabilistic Programming</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>9437</v>
+      </c>
+      <c r="E45" t="n">
+        <v>7</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>2</v>
+      </c>
+      <c r="L45" t="n">
+        <v>4</v>
+      </c>
+      <c r="M45" t="n">
+        <v>25</v>
+      </c>
+      <c r="N45" t="n">
+        <v>266</v>
+      </c>
+      <c r="O45" t="n">
+        <v>18</v>
+      </c>
+      <c r="P45" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Overview, 1. From explicit Bayes to declarative Bayes, 2. Anatomy of a probabilistic program, 3. Constrained-to-unconstrained transforms, 4. Inference dispatch: NUTS, ADVI, and MAP, 5. The Bayesian workflow on eight schools, 6. Limits, alternatives, and connections</t>
         </is>
       </c>
     </row>
@@ -4156,16 +4230,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>5752</v>
+        <v>6980</v>
       </c>
       <c r="D11" t="n">
         <v>2764</v>
       </c>
       <c r="E11" t="n">
-        <v>8739</v>
+        <v>9437</v>
       </c>
       <c r="F11" t="n">
         <v>7</v>
@@ -4177,10 +4251,10 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" t="n">
         <v>2</v>
-      </c>
-      <c r="J11" t="n">
-        <v>1</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -4200,7 +4274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5505,6 +5579,33 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Probabilistic Programming</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>bayesian-ml</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Missing code section</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Code lives in the verified notebook at notebooks/probabilistic-programming/01_probabilistic_programming.ipynb (PyMC 5 + NumPyro for §§1, 3, 4, 5 fit-and-sample cells; Stan shown statically in §2.4 only). The MDX walks the computational story in §1.2, §2.4, and §5.3 with three short pedagogical code blocks (PyMC Beta–Binomial declaration, Stan model in `data`/`parameters`/`model` blocks, and the centered-vs-non-centered diff) but no dedicated Computational Notes section.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(bnn): regenerate cross-site audit artifacts and content metrics
audit-output/formalml-references.json, cross-site-audit-report.md, and
deferred-reciprocals.md regenerated by pnpm audit:cross-site after BNN
landed. The audit recognizes BNN's six cross-site edges (5 formalstatistics
prereqs + 1 formalcalculus prereq) and slots them into "Missing reciprocals"
on the formalstatistics → formalml side — these become sister-site PRs to
discharge:
  - formalstatistics/bayesian-foundations-and-prior-selection
  - formalstatistics/central-limit-theorem
  - formalstatistics/modes-of-convergence
  - formalstatistics/multivariate-distributions
  - formalstatistics/hierarchical-bayes-and-partial-pooling
  - formalcalculus/jacobian

No self-site warnings, no slug-drift candidates after the jacobians→jacobian
fix. No direction mismatches.

Content metrics spreadsheet updated by prior session with the BNN row in
Topic Detail.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R46"/>
+  <dimension ref="A1:R47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3855,6 +3855,80 @@
       <c r="R46" t="inlineStr">
         <is>
           <t>Overview, 1. Three responses to grouped data, 2. The linear mixed model, 3. Henderson's mixed-model equations and BLUP, 4. REML for variance components, 5. The frequentist–Bayesian bridge, 6. Connections, limits, and references</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>bayesian-ml</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Bayesian Neural Networks</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>11882</v>
+      </c>
+      <c r="E47" t="n">
+        <v>11</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="n">
+        <v>46</v>
+      </c>
+      <c r="M47" t="n">
+        <v>68</v>
+      </c>
+      <c r="N47" t="n">
+        <v>730</v>
+      </c>
+      <c r="O47" t="n">
+        <v>24</v>
+      </c>
+      <c r="P47" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0</v>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Overview, 1. Why Bayesian over the weights, 2. The weight-space posterior, 3. The Laplace approximation, 4. MC-dropout as approximate variational inference, 5. Deep ensembles as a function-space posterior proxy, 6. Stochastic-gradient Langevin dynamics (SGLD), 7. Stochastic-gradient HMC (SGHMC), 8. Calibration and uncertainty quantification, 9. Function-space view: NNGP, NTK, and open problems, Connections and further reading</t>
         </is>
       </c>
     </row>
@@ -4304,19 +4378,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>7396</v>
+        <v>8293</v>
       </c>
       <c r="D11" t="n">
         <v>2764</v>
       </c>
       <c r="E11" t="n">
-        <v>9437</v>
+        <v>11882</v>
       </c>
       <c r="F11" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="G11" t="n">
         <v>1</v>
@@ -4325,7 +4399,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J11" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
docs(content-metrics): add high-dimensional-regression row; T2 published 2 → 3
Topic Detail row 51:
- supervised-learning · High-Dimensional Regression · advanced
- 17,945 words, 12 sections, 24 TheoremBlocks, 49 display eqs, 229 inline math
- 50 references, all with URLs (0 missing)
- All content-quality flags Yes

Domain Summary supervised-learning rollup:
- Topics: 2 → 3
- Avg words: 6977 → 10633 (high-dim is roughly 2× kernel-regression / local-regression
  due to denser theory + 12 sections vs 10-13)
- Min/Max words: 6856 / 17945
- All gap-metric columns remain 0 (high-dim clears every threshold)

No Gap Analysis entries added — topic exceeds 3k words, has ≥7 sections, has
code-section (notebook), has viz, has connections.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R50"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4151,6 +4151,80 @@
       <c r="R50" t="inlineStr">
         <is>
           <t>1. From local-linear to degree-$p$ | 2. The degree-$p$ local polynomial estimator | 3. The equivalent-kernel formulation | 4. Bias and variance at general $p$ | 5. The boundary and the odd-vs-even degree story | 6. Boundary behavior across the full support | 7. Bandwidth selection at general $p$ | 8. Multivariate local polynomials | 9. Derivative estimation | 10. Connections to smoothing splines | 11. Connections to additive models | 12. Connections, applications, and limits | Connections and Further Reading</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>supervised-learning</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>High-Dimensional Regression</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>17945</v>
+      </c>
+      <c r="E51" t="n">
+        <v>12</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="n">
+        <v>24</v>
+      </c>
+      <c r="M51" t="n">
+        <v>49</v>
+      </c>
+      <c r="N51" t="n">
+        <v>229</v>
+      </c>
+      <c r="O51" t="n">
+        <v>50</v>
+      </c>
+      <c r="P51" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>1. From OLS to penalized regression | 2. The lasso estimator | 3. Solving the lasso | 4. Bias-variance for the lasso | 5. The lasso oracle inequality | 6. Variable-selection consistency | 7. Cross-validation for λ | 8. Ridge, elastic net, and adaptive lasso | 9. Geometry of the high-dimensional regime | 10. Post-selection inference and the debiased lasso | 11. Generalized lasso for non-Gaussian responses | 12. Connections, applications, and limits</t>
         </is>
       </c>
     </row>
@@ -4640,19 +4714,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>6977</v>
+        <v>10633</v>
       </c>
       <c r="D12" t="n">
         <v>6856</v>
       </c>
       <c r="E12" t="n">
-        <v>7098</v>
+        <v>17945</v>
       </c>
       <c r="F12" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
docs(content-metrics): add generalization-bounds row; T6 learning-theory 0 → 1 published
Row metrics: 13,112 words, 14 H2 sections, 43 theorem blocks, 68 display
equations, 25 references all with URLs.  New Domain Summary row for
"learning-theory" with the inaugural-topic baseline.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R52"/>
+  <dimension ref="A1:R53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4299,6 +4299,80 @@
       <c r="R52" t="inlineStr">
         <is>
           <t>Motivation: explicit-density generative models, Change of variables in d dimensions, The normalizing-flow framework, Coupling layers — NICE and RealNVP, Autoregressive flows — MAF and IAF, Multi-scale and image-domain architectures, Maximum-likelihood training, Expressivity and universality, Flows for variational inference, Flows for density estimation, Worked example: 2-moons end-to-end, Connections, applications, and limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>learning-theory</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Generalization Bounds</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>13112</v>
+      </c>
+      <c r="E53" t="n">
+        <v>14</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="n">
+        <v>43</v>
+      </c>
+      <c r="M53" t="n">
+        <v>68</v>
+      </c>
+      <c r="N53" t="n">
+        <v>875</v>
+      </c>
+      <c r="O53" t="n">
+        <v>25</v>
+      </c>
+      <c r="P53" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>0</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Motivation: why bound the generalization gap?, The generalization gap and its decomposition, Finite-class warmup, Uniform convergence and Glivenko–Cantelli, Rademacher complexity, Symmetrization, McDiarmid + Rademacher → uniform convergence, Real-valued function classes, Data-dependent bounds, Margin bounds, Algorithmic stability bounds, Worked example: empirical Rademacher and vacuousness, Computational notes, Connections and limits</t>
         </is>
       </c>
     </row>
@@ -4313,7 +4387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4858,6 +4932,46 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>learning-theory</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>13112</v>
+      </c>
+      <c r="D14" t="n">
+        <v>13112</v>
+      </c>
+      <c r="E14" t="n">
+        <v>13112</v>
+      </c>
+      <c r="F14" t="n">
+        <v>14</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(pac-bayes-bounds): topic MDX + 12 viz + Dziugaite–Roy reproduction
Ships the second T6 Learning Theory topic. Develops PAC-Bayes from first
principles via Donsker–Varadhan + McAllester / Seeger / Catoni and closes
with a NumPy-only Dziugaite–Roy reproduction certifying 0.2369 on a
~13k-parameter MLP at binary MNIST — well below the vacuous Rademacher
floor of 1. Discharges the deferred formalstatistics/empirical-processes
reciprocal pointer.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R53"/>
+  <dimension ref="A1:R54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4373,6 +4373,80 @@
       <c r="R53" t="inlineStr">
         <is>
           <t>Motivation: why bound the generalization gap?, The generalization gap and its decomposition, Finite-class warmup, Uniform convergence and Glivenko–Cantelli, Rademacher complexity, Symmetrization, McDiarmid + Rademacher → uniform convergence, Real-valued function classes, Data-dependent bounds, Margin bounds, Algorithmic stability bounds, Worked example: empirical Rademacher and vacuousness, Computational notes, Connections and limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>learning-theory</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PAC-Bayes Bounds</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>8107</v>
+      </c>
+      <c r="E54" t="n">
+        <v>14</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>1</v>
+      </c>
+      <c r="L54" t="n">
+        <v>11</v>
+      </c>
+      <c r="M54" t="n">
+        <v>76</v>
+      </c>
+      <c r="N54" t="n">
+        <v>763</v>
+      </c>
+      <c r="O54" t="n">
+        <v>43</v>
+      </c>
+      <c r="P54" t="n">
+        <v>43</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Motivation: beyond uniform convergence, The PAC-Bayes setup, The change-of-measure inequality, The McAllester bound, The Seeger / kl-form bound, The Catoni / linear bound and the Gibbs posterior, Refinements, Choosing prior and posterior in continuous classes, The Bayesian–PAC-Bayes correspondence, Three bounds on the running example, Non-vacuous deep-network bounds (Dziugaite–Roy 2017), ML applications, Computational notes, Connections and limits</t>
         </is>
       </c>
     </row>
@@ -4942,13 +5016,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>13112</v>
+        <v>10609.5</v>
       </c>
       <c r="D14" t="n">
-        <v>13112</v>
+        <v>8107</v>
       </c>
       <c r="E14" t="n">
         <v>13112</v>

</xml_diff>

<commit_message>
chore(clustering): content-metrics spreadsheet row + domain rollup
  - Topic Detail: row 61 added — domain=unsupervised, words=6346,
    sections=12, all five content flags Yes, python blocks=1,
    theorem blocks=20, display eqs=37, inline math=524, refs total=41,
    refs w/ URL=41, refs missing URL=0.
  - Domain Summary: unsupervised row recomputed — 2 topics (clustering
    + normalizing-flows), avg 10198 words, avg 12 sections, 0 refs
    missing URL across the domain.
  - Gap Analysis: clustering meets all thresholds (12 sections > 7,
    6346 words > 3k, has code section) — no entry needed.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R60"/>
+  <dimension ref="A1:R61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4891,6 +4891,80 @@
       <c r="R60" t="inlineStr">
         <is>
           <t>Motivation, Tangent spaces, Efficient influence functions, Semiparametric efficiency bound, One-step estimators, Targeted maximum likelihood (TMLE), Double / debiased machine learning (DML), Sample-splitting and cross-fitting, Worked examples, Inference and confidence intervals, Connections to uncertainty quantification, Connections to causal inference, Computational notes, Connections and limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>unsupervised</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Clustering</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>6346</v>
+      </c>
+      <c r="E61" t="n">
+        <v>12</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>1</v>
+      </c>
+      <c r="L61" t="n">
+        <v>20</v>
+      </c>
+      <c r="M61" t="n">
+        <v>37</v>
+      </c>
+      <c r="N61" t="n">
+        <v>524</v>
+      </c>
+      <c r="O61" t="n">
+        <v>41</v>
+      </c>
+      <c r="P61" t="n">
+        <v>41</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Motivation: when linear partitions fail, The KDE substrate and the mode-finding picture, Mean-shift as gradient ascent on f_h, Convergence theory, Bandwidth resolution and the mode tree, Kernel-function choice, From trajectories to clusters, Practical mean-shift, k-means as the h-to-0 Voronoi limit, GMM-via-EM and soft assignment, Pointers: spectral and density-based clustering, Connections limits and forward pointers</t>
         </is>
       </c>
     </row>
@@ -5420,13 +5494,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" t="n">
-        <v>14049</v>
+        <v>10197.5</v>
       </c>
       <c r="D13" t="n">
-        <v>14049</v>
+        <v>6346</v>
       </c>
       <c r="E13" t="n">
         <v>14049</v>

</xml_diff>

<commit_message>
docs(riemann-manifold-hmc): update content metrics spreadsheet
Topic Detail: new row for Riemann Manifold HMC.
  Domain: bayesian-ml | Difficulty: advanced
  Words: 10,714 | Sections: 12
  Python blocks: 2 | TheoremBlocks: 11 | Display Eqs: 53 | Inline Math: 671
  Refs: 22 / 22 / 0 (total / with URL / missing)

Domain Summary: bayesian-ml row recomputed across the topics currently
in the sheet (sheet contains a subset of shipped bayesian-ml topics —
the previous 10-topic count from the strategic-planning narrative is
an authorial roll-up, not the spreadsheet's row count).

Gap Analysis: no new rows for RMHMC (10k words > 3k threshold, 12
sections > 7 threshold, has code section).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topic Detail" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R61"/>
+  <dimension ref="A1:R62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -827,24 +827,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>topology</t>
+          <t>bayesian-ml</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Čech Complexes &amp; Nerve Theorem</t>
+          <t>Riemann Manifold HMC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>861</v>
+        <v>10714</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -872,41 +872,41 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="M6" t="n">
-        <v>10</v>
+        <v>53</v>
       </c>
       <c r="N6" t="n">
-        <v>207</v>
+        <v>671</v>
       </c>
       <c r="O6" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="P6" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, The Čech Complex, The Nerve of a Cover, The Nerve Theorem, Čech vs. Vietoris-Rips: The Interleaving Inequality, The Phantom Cycle: A Detailed Analysis, Computational Comparison, Applications &amp; Connections</t>
+          <t>§1. Overview &amp; Motivation, §2. HMC at a glance, §3. Riemannian geometry of probability, §4. The Riemannian Hamiltonian, §5. The Generalized Leapfrog Integrator, §6. Volume preservation, reversibility, and detailed balance, §7. Step size, trajectory length, and ergodicity, §8. Computational cost, §9. Worked example: the banana distribution, §10. Worked example: log-Gaussian Cox process, §11. Computational notes, §12. Connections and limits</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>probability</t>
+          <t>topology</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Concentration Inequalities</t>
+          <t>Čech Complexes &amp; Nerve Theorem</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -915,10 +915,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>808</v>
+        <v>861</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -946,41 +946,41 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L7" t="n">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="M7" t="n">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="N7" t="n">
-        <v>280</v>
+        <v>207</v>
       </c>
       <c r="O7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Basic Tail Bounds: Markov and Chebyshev, The Chernoff Method and Moment Generating Functions, Hoeffding's Inequality, Sub-Gaussian Random Variables, Sub-Exponential Random Variables and Bernstein's Inequality, McDiarmid's Inequality, Applications to Machine Learning, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, The Čech Complex, The Nerve of a Cover, The Nerve Theorem, Čech vs. Vietoris-Rips: The Interleaving Inequality, The Phantom Cycle: A Detailed Analysis, Computational Comparison, Applications &amp; Connections</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>nonparametric-ml</t>
+          <t>probability</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Conformal Prediction</t>
+          <t>Concentration Inequalities</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -989,19 +989,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3386</v>
+        <v>808</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1020,67 +1020,67 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L8" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="M8" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="N8" t="n">
-        <v>468</v>
+        <v>280</v>
       </c>
       <c r="O8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q8" t="n">
         <v>0</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Distribution-Free Prediction and the Exchangeability Setup, Split (Inductive) Conformal Prediction, Marginal Coverage: The Central Theorem, Full (Transductive) Conformal Prediction, Jackknife+ and CV+, Conformalized Quantile Regression (CQR), Adaptive Prediction Sets (APS) for Classification, Conditional Coverage: Impossibility and Approximations, Wrapping Black-Box ML Models, Notation Reference, Forward Connections to Planned formalML Topics</t>
+          <t>Overview &amp; Motivation, Basic Tail Bounds: Markov and Chebyshev, The Chernoff Method and Moment Generating Functions, Hoeffding's Inequality, Sub-Gaussian Random Variables, Sub-Exponential Random Variables and Bernstein's Inequality, McDiarmid's Inequality, Applications to Machine Learning, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>optimization</t>
+          <t>nonparametric-ml</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Convex Analysis</t>
+          <t>Conformal Prediction</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>foundational</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2284</v>
+        <v>3386</v>
       </c>
       <c r="E9" t="n">
         <v>11</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1094,50 +1094,50 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="M9" t="n">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="N9" t="n">
-        <v>253</v>
+        <v>468</v>
       </c>
       <c r="O9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="P9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="Q9" t="n">
         <v>0</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Convex Sets, Convex Hull &amp; Extreme Points, Convex Functions, First-Order &amp; Second-Order Conditions, Operations Preserving Convexity, Conjugate Functions, Subdifferentials &amp; Subgradients, Separation Theorems, Computational Notes, Connections &amp; Further Reading</t>
+          <t>Distribution-Free Prediction and the Exchangeability Setup, Split (Inductive) Conformal Prediction, Marginal Coverage: The Central Theorem, Full (Transductive) Conformal Prediction, Jackknife+ and CV+, Conformalized Quantile Regression (CQR), Adaptive Prediction Sets (APS) for Classification, Conditional Coverage: Impossibility and Approximations, Wrapping Black-Box ML Models, Notation Reference, Forward Connections to Planned formalML Topics</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>graph-theory</t>
+          <t>optimization</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Expander Graphs</t>
+          <t>Convex Analysis</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>foundational</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1958</v>
+        <v>2284</v>
       </c>
       <c r="E10" t="n">
         <v>11</v>
@@ -1168,16 +1168,16 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L10" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="M10" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="N10" t="n">
-        <v>693</v>
+        <v>253</v>
       </c>
       <c r="O10" t="n">
         <v>6</v>
@@ -1190,35 +1190,35 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, 1. Three Notions of Expansion, 2. The Relationship Between Expansion Notions, 3. Cheeger's Inequality: Linking Spectrum to Combinatorics, 4. The Expander Mixing Lemma, 5. Ramanujan Graphs and the Alon-Boppana Bound, 6. Explicit Constructions, 7. Random Walks on Expanders, 8. Applications to Computer Science and Machine Learning, 9. Computational Notes, 10. Connections and Further Reading</t>
+          <t>Overview &amp; Motivation, Convex Sets, Convex Hull &amp; Extreme Points, Convex Functions, First-Order &amp; Second-Order Conditions, Operations Preserving Convexity, Conjugate Functions, Subdifferentials &amp; Subgradients, Separation Theorems, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>nonparametric-ml</t>
+          <t>graph-theory</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Extreme Value Theory</t>
+          <t>Expander Graphs</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4976</v>
+        <v>1958</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1242,57 +1242,57 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L11" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="M11" t="n">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="N11" t="n">
-        <v>1137</v>
+        <v>693</v>
       </c>
       <c r="O11" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="P11" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1. From the center to the tails, 2. Max-stability and the Fisher–Tippett–Gnedenko trichotomy, 3. Domains of attraction, 4. Block-maxima inference, 5. Peaks over threshold and the generalized Pareto distribution, 6. Connections, ML applications, and limits, Connections and Further Reading</t>
+          <t>Overview &amp; Motivation, 1. Three Notions of Expansion, 2. The Relationship Between Expansion Notions, 3. Cheeger's Inequality: Linking Spectrum to Combinatorics, 4. The Expander Mixing Lemma, 5. Ramanujan Graphs and the Alon-Boppana Bound, 6. Explicit Constructions, 7. Random Walks on Expanders, 8. Applications to Computer Science and Machine Learning, 9. Computational Notes, 10. Connections and Further Reading</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>geometry</t>
+          <t>nonparametric-ml</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Geodesics &amp; Curvature</t>
+          <t>Extreme Value Theory</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2160</v>
+        <v>4976</v>
       </c>
       <c r="E12" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1316,41 +1316,41 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M12" t="n">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="N12" t="n">
-        <v>358</v>
+        <v>1137</v>
       </c>
       <c r="O12" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="P12" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="Q12" t="n">
         <v>0</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Geodesics: Curves of Zero Acceleration, The Exponential Map &amp; Normal Coordinates, The Riemann Curvature Tensor, Sectional, Ricci, and Scalar Curvature, The Gauss–Bonnet Theorem, Jacobi Fields &amp; Geodesic Deviation, Comparison Theorems, Computational Notes, Connections to Machine Learning, Connections &amp; Further Reading</t>
+          <t>1. From the center to the tails, 2. Max-stability and the Fisher–Tippett–Gnedenko trichotomy, 3. Domains of attraction, 4. Block-maxima inference, 5. Peaks over threshold and the generalized Pareto distribution, 6. Connections, ML applications, and limits, Connections and Further Reading</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>optimization</t>
+          <t>geometry</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Gradient Descent &amp; Convergence</t>
+          <t>Geodesics &amp; Curvature</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1359,10 +1359,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2491</v>
+        <v>2160</v>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1390,53 +1390,53 @@
         </is>
       </c>
       <c r="K13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" t="n">
+        <v>29</v>
+      </c>
+      <c r="M13" t="n">
+        <v>23</v>
+      </c>
+      <c r="N13" t="n">
+        <v>358</v>
+      </c>
+      <c r="O13" t="n">
         <v>6</v>
       </c>
-      <c r="L13" t="n">
-        <v>27</v>
-      </c>
-      <c r="M13" t="n">
-        <v>47</v>
-      </c>
-      <c r="N13" t="n">
-        <v>263</v>
-      </c>
-      <c r="O13" t="n">
-        <v>7</v>
-      </c>
       <c r="P13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, The Gradient Descent Algorithm, Smoothness &amp; the Descent Lemma, Convergence for Convex Functions, Strong Convexity &amp; Linear Convergence, Step Size Selection, Nesterov Accelerated Gradient, Coordinate Descent, Mirror Descent &amp; Bregman Divergence, Stochastic Gradient Descent, Computational Notes, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, Geodesics: Curves of Zero Acceleration, The Exponential Map &amp; Normal Coordinates, The Riemann Curvature Tensor, Sectional, Ricci, and Scalar Curvature, The Gauss–Bonnet Theorem, Jacobi Fields &amp; Geodesic Deviation, Comparison Theorems, Computational Notes, Connections to Machine Learning, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>graph-theory</t>
+          <t>optimization</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Graph Laplacians &amp; Spectrum</t>
+          <t>Gradient Descent &amp; Convergence</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>foundational</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1491</v>
+        <v>2491</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1464,53 +1464,53 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L14" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="M14" t="n">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="N14" t="n">
-        <v>316</v>
+        <v>263</v>
       </c>
       <c r="O14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Graphs, Adjacency Matrices, and the Degree Matrix, The Graph Laplacian, Spectral Properties of the Laplacian, The Normalized Laplacian, Cheeger's Inequality, Spectral Clustering, Connections to Machine Learning, Computational Notes, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, The Gradient Descent Algorithm, Smoothness &amp; the Descent Lemma, Convergence for Convex Functions, Strong Convexity &amp; Linear Convergence, Step Size Selection, Nesterov Accelerated Gradient, Coordinate Descent, Mirror Descent &amp; Bregman Divergence, Stochastic Gradient Descent, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>geometry</t>
+          <t>graph-theory</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Information Geometry &amp; Fisher Metric</t>
+          <t>Graph Laplacians &amp; Spectrum</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>foundational</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3953</v>
+        <v>1491</v>
       </c>
       <c r="E15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1538,53 +1538,53 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L15" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="M15" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="N15" t="n">
-        <v>271</v>
+        <v>316</v>
       </c>
       <c r="O15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Statistical Manifolds &amp; Parametric Families, The Fisher Information Metric, Fisher Metric for Classical Families, $\alpha$-Connections and Dual Geometry, Divergence Functions, Geodesics on Statistical Manifolds, The Cramér–Rao Bound, Computational Notes, Information Geometry in Machine Learning, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, Graphs, Adjacency Matrices, and the Degree Matrix, The Graph Laplacian, Spectral Properties of the Laplacian, The Normalized Laplacian, Cheeger's Inequality, Spectral Clustering, Connections to Machine Learning, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>information-theory</t>
+          <t>geometry</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>KL Divergence &amp; f-Divergences</t>
+          <t>Information Geometry &amp; Fisher Metric</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1085</v>
+        <v>3953</v>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1612,16 +1612,16 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L16" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="M16" t="n">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="N16" t="n">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="O16" t="n">
         <v>7</v>
@@ -1634,31 +1634,31 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, KL Divergence: Definition &amp; Properties, Forward vs Reverse KL, f-Divergences: A Unifying Framework, Properties of f-Divergences, Variational Representations, Rényi Divergence &amp; $\alpha$-Divergences, Computational Notes, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, Statistical Manifolds &amp; Parametric Families, The Fisher Information Metric, Fisher Metric for Classical Families, $\alpha$-Connections and Dual Geometry, Divergence Functions, Geodesics on Statistical Manifolds, The Cramér–Rao Bound, Computational Notes, Information Geometry in Machine Learning, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>optimization</t>
+          <t>information-theory</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Lagrangian Duality &amp; KKT Conditions</t>
+          <t>KL Divergence &amp; f-Divergences</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>906</v>
+        <v>1085</v>
       </c>
       <c r="E17" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1686,41 +1686,41 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L17" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M17" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="N17" t="n">
-        <v>282</v>
+        <v>266</v>
       </c>
       <c r="O17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, The Lagrangian &amp; Dual Problem, Weak Duality, Strong Duality &amp; Slater's Condition, KKT Conditions, Complementary Slackness, Saddle Point Interpretation, Sensitivity Analysis, Application: The SVM Dual, Application: Water-Filling &amp; Portfolio Optimization, Computational Notes, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, KL Divergence: Definition &amp; Properties, Forward vs Reverse KL, f-Divergences: A Unifying Framework, Properties of f-Divergences, Variational Representations, Rényi Divergence &amp; $\alpha$-Divergences, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>topology</t>
+          <t>optimization</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>The Mapper Algorithm</t>
+          <t>Lagrangian Duality &amp; KKT Conditions</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1729,7 +1729,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3215</v>
+        <v>906</v>
       </c>
       <c r="E18" t="n">
         <v>12</v>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1760,124 +1760,124 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L18" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="M18" t="n">
+        <v>31</v>
+      </c>
+      <c r="N18" t="n">
+        <v>282</v>
+      </c>
+      <c r="O18" t="n">
         <v>6</v>
       </c>
-      <c r="N18" t="n">
-        <v>119</v>
-      </c>
-      <c r="O18" t="n">
-        <v>8</v>
-      </c>
       <c r="P18" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, The Mapper Pipeline, Interactive Pipeline Explorer, Filter Functions, Covering &amp; Pullback, From-Scratch Implementation, Classic Examples, KeplerMapper, Parameter Sensitivity, The Nerve Theorem Connection, Financial Market Regime Detection, Stability &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, The Lagrangian &amp; Dual Problem, Weak Duality, Strong Duality &amp; Slater's Condition, KKT Conditions, Complementary Slackness, Saddle Point Interpretation, Sensitivity Analysis, Application: The SVM Dual, Application: Water-Filling &amp; Portfolio Optimization, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>probability</t>
+          <t>topology</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Measure-Theoretic Probability</t>
+          <t>The Mapper Algorithm</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1209</v>
+        <v>3215</v>
       </c>
       <c r="E19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>7</v>
+      </c>
+      <c r="L19" t="n">
         <v>10</v>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L19" t="n">
-        <v>66</v>
-      </c>
       <c r="M19" t="n">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="N19" t="n">
-        <v>471</v>
+        <v>119</v>
       </c>
       <c r="O19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q19" t="n">
         <v>0</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Sigma-Algebras and Measurable Spaces, Measures and Probability Measures, Measurable Functions and Random Variables, The Lebesgue Integral and Expectation, Convergence of Random Variables, Product Measures and Fubini's Theorem, Conditional Expectation and Radon–Nikodym, A Preview of Martingales, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, The Mapper Pipeline, Interactive Pipeline Explorer, Filter Functions, Covering &amp; Pullback, From-Scratch Implementation, Classic Examples, KeplerMapper, Parameter Sensitivity, The Nerve Theorem Connection, Financial Market Regime Detection, Stability &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>graph-theory</t>
+          <t>probability</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Message Passing &amp; GNNs</t>
+          <t>Measure-Theoretic Probability</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2619</v>
+        <v>1209</v>
       </c>
       <c r="E20" t="n">
         <v>10</v>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1911,38 +1911,38 @@
         <v>3</v>
       </c>
       <c r="L20" t="n">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="M20" t="n">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="N20" t="n">
-        <v>191</v>
+        <v>471</v>
       </c>
       <c r="O20" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="P20" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q20" t="n">
         <v>0</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, The Message Passing Framework, Spectral Graph Convolutions, Spatial Graph Convolutions, The Weisfeiler-Leman Test &amp; GNN Expressiveness, Attention-Based Message Passing, Over-Smoothing &amp; the Random Walk Connection, Expander-Based Graph Rewiring, Computational Notes, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, Sigma-Algebras and Measurable Spaces, Measures and Probability Measures, Measurable Functions and Random Variables, The Lebesgue Integral and Expectation, Convergence of Random Variables, Product Measures and Fubini's Theorem, Conditional Expectation and Radon–Nikodym, A Preview of Martingales, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>information-theory</t>
+          <t>graph-theory</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Minimum Description Length</t>
+          <t>Message Passing &amp; GNNs</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2250</v>
+        <v>2619</v>
       </c>
       <c r="E21" t="n">
         <v>10</v>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1982,41 +1982,41 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L21" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="M21" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="N21" t="n">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="O21" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="P21" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="Q21" t="n">
         <v>0</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Two-Part Codes &amp; Crude MDL, Kolmogorov Complexity, Stochastic Complexity &amp; Refined MDL, Fisher Information &amp; Asymptotic Complexity, MDL and Bayesian Model Selection, Prequential Codes &amp; Online MDL, MDL for Practical Model Selection, Computational Notes, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, The Message Passing Framework, Spectral Graph Convolutions, Spatial Graph Convolutions, The Weisfeiler-Leman Test &amp; GNN Expressiveness, Attention-Based Message Passing, Over-Smoothing &amp; the Random Walk Connection, Expander-Based Graph Rewiring, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>category-theory</t>
+          <t>information-theory</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Monads &amp; Comonads</t>
+          <t>Minimum Description Length</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2025,10 +2025,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2564</v>
+        <v>2250</v>
       </c>
       <c r="E22" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -2056,29 +2056,29 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="M22" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="N22" t="n">
-        <v>343</v>
+        <v>189</v>
       </c>
       <c r="O22" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="P22" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="Q22" t="n">
         <v>0</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Overview and Motivation, Monads: Definition and Laws, From Adjunctions to Monads, A Gallery of Monads, Kleisli Categories, Markov Kernels and the Giry Monad, Eilenberg-Moore Algebras, Two Canonical Adjunctions, Beck's Monadicity Theorem, Comonads, Monad-Comonad Duality, A Gallery of Comonads, Monads and Comonads in Machine Learning, Computational Notes, Connections and Further Reading</t>
+          <t>Overview &amp; Motivation, Two-Part Codes &amp; Crude MDL, Kolmogorov Complexity, Stochastic Complexity &amp; Refined MDL, Fisher Information &amp; Asymptotic Complexity, MDL and Bayesian Model Selection, Prequential Codes &amp; Online MDL, MDL for Practical Model Selection, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
@@ -2090,90 +2090,90 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Natural Transformations</t>
+          <t>Monads &amp; Comonads</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2250</v>
+        <v>2564</v>
       </c>
       <c r="E23" t="n">
+        <v>15</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>4</v>
+      </c>
+      <c r="L23" t="n">
+        <v>21</v>
+      </c>
+      <c r="M23" t="n">
+        <v>8</v>
+      </c>
+      <c r="N23" t="n">
+        <v>343</v>
+      </c>
+      <c r="O23" t="n">
         <v>10</v>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K23" t="n">
-        <v>3</v>
-      </c>
-      <c r="L23" t="n">
-        <v>24</v>
-      </c>
-      <c r="M23" t="n">
-        <v>17</v>
-      </c>
-      <c r="N23" t="n">
-        <v>330</v>
-      </c>
-      <c r="O23" t="n">
-        <v>6</v>
-      </c>
       <c r="P23" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Natural Transformations: Morphisms Between Functors, A Gallery of Natural Transformations, Composition of Natural Transformations, Functor Categories, The Yoneda Lemma, The Yoneda Embedding and Presheaves, Equivariance as Naturality, Computational Notes, Connections &amp; Further Reading</t>
+          <t>Overview and Motivation, Monads: Definition and Laws, From Adjunctions to Monads, A Gallery of Monads, Kleisli Categories, Markov Kernels and the Giry Monad, Eilenberg-Moore Algebras, Two Canonical Adjunctions, Beck's Monadicity Theorem, Comonads, Monad-Comonad Duality, A Gallery of Comonads, Monads and Comonads in Machine Learning, Computational Notes, Connections and Further Reading</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>probability</t>
+          <t>category-theory</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PAC Learning Framework</t>
+          <t>Natural Transformations</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1290</v>
+        <v>2250</v>
       </c>
       <c r="E24" t="n">
         <v>10</v>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2204,53 +2204,53 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L24" t="n">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="M24" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="N24" t="n">
-        <v>416</v>
+        <v>330</v>
       </c>
       <c r="O24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q24" t="n">
         <v>0</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, The Learning Problem, Realizable PAC Learning, Agnostic PAC Learning, The VC Dimension, Sauer–Shelah Lemma and Growth Functions, The Fundamental Theorem of Statistical Learning, Rademacher Complexity, Applications and Worked Examples, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, Natural Transformations: Morphisms Between Functors, A Gallery of Natural Transformations, Composition of Natural Transformations, Functor Categories, The Yoneda Lemma, The Yoneda Embedding and Presheaves, Equivariance as Naturality, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>linear-algebra</t>
+          <t>probability</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PCA &amp; Low-Rank Approximation</t>
+          <t>PAC Learning Framework</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>761</v>
+        <v>1290</v>
       </c>
       <c r="E25" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -2278,41 +2278,41 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L25" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="M25" t="n">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="N25" t="n">
-        <v>191</v>
+        <v>416</v>
       </c>
       <c r="O25" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="P25" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="Q25" t="n">
         <v>0</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, PCA from First Principles: Variance Maximization, PCA via the SVD, Geometric Interpretation, The Scree Plot and Dimensionality Selection, Low-Rank Approximation as Optimal Projection, Computing PCA in Practice, Application: High-Dimensional Data Visualization, Kernel PCA, Probabilistic PCA, Robust PCA: Principal Component Pursuit, Sparse PCA, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, The Learning Problem, Realizable PAC Learning, Agnostic PAC Learning, The VC Dimension, Sauer–Shelah Lemma and Growth Functions, The Fundamental Theorem of Statistical Learning, Rademacher Complexity, Applications and Worked Examples, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>topology</t>
+          <t>linear-algebra</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Persistent Homology</t>
+          <t>PCA &amp; Low-Rank Approximation</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2321,10 +2321,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>3878</v>
+        <v>761</v>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -2333,12 +2333,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2355,38 +2355,38 @@
         <v>6</v>
       </c>
       <c r="L26" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="M26" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N26" t="n">
-        <v>287</v>
+        <v>191</v>
       </c>
       <c r="O26" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="P26" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q26" t="n">
         <v>0</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Formal Framework, The Matrix Reduction Algorithm, Visual Intuition, The Stability Theorem, Extended Persistence, Persistence Modules, Working Code, Connections &amp; Cross-Track Bridges, Exercises</t>
+          <t>Overview &amp; Motivation, PCA from First Principles: Variance Maximization, PCA via the SVD, Geometric Interpretation, The Scree Plot and Dimensionality Selection, Low-Rank Approximation as Optimal Projection, Computing PCA in Practice, Application: High-Dimensional Data Visualization, Kernel PCA, Probabilistic PCA, Robust PCA: Principal Component Pursuit, Sparse PCA, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>nonparametric-ml</t>
+          <t>topology</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Prediction Intervals</t>
+          <t>Persistent Homology</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2395,72 +2395,72 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8089</v>
+        <v>3878</v>
       </c>
       <c r="E27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>6</v>
+      </c>
+      <c r="L27" t="n">
+        <v>30</v>
+      </c>
+      <c r="M27" t="n">
+        <v>18</v>
+      </c>
+      <c r="N27" t="n">
+        <v>287</v>
+      </c>
+      <c r="O27" t="n">
         <v>7</v>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="n">
-        <v>22</v>
-      </c>
-      <c r="M27" t="n">
-        <v>42</v>
-      </c>
-      <c r="N27" t="n">
-        <v>623</v>
-      </c>
-      <c r="O27" t="n">
-        <v>15</v>
-      </c>
       <c r="P27" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="Q27" t="n">
         <v>0</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>The Prediction-Interval Problem, Construction I — Exchangeability-Based (Split Conformal), Construction II — Conditional-Quantile (Pure QR Intervals), Construction III — Test-Inversion (HL-Style Prediction Intervals), Bridge Theorems, Empirical Comparison: Coverage, Width, Conditional Behavior, Cost, Limits, Connections, and What's Out of Scope</t>
+          <t>Overview &amp; Motivation, Formal Framework, The Matrix Reduction Algorithm, Visual Intuition, The Stability Theorem, Extended Persistence, Persistence Modules, Working Code, Connections &amp; Cross-Track Bridges, Exercises</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>optimization</t>
+          <t>nonparametric-ml</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Proximal Methods</t>
+          <t>Prediction Intervals</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2469,24 +2469,24 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>965</v>
+        <v>8089</v>
       </c>
       <c r="E28" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2500,41 +2500,41 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="M28" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="N28" t="n">
-        <v>312</v>
+        <v>623</v>
       </c>
       <c r="O28" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="P28" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="Q28" t="n">
         <v>0</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, The Proximal Operator, Proximal Operator Catalog, The Moreau Envelope, Proximal Gradient Descent, ISTA &amp; Soft-Thresholding, FISTA: Accelerated Proximal Gradient, Douglas–Rachford Splitting, ADMM, Convergence Analysis, Computational Notes, Connections &amp; Further Reading</t>
+          <t>The Prediction-Interval Problem, Construction I — Exchangeability-Based (Split Conformal), Construction II — Conditional-Quantile (Pure QR Intervals), Construction III — Test-Inversion (HL-Style Prediction Intervals), Bridge Theorems, Empirical Comparison: Coverage, Width, Conditional Behavior, Cost, Limits, Connections, and What's Out of Scope</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>nonparametric-ml</t>
+          <t>optimization</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Quantile Regression</t>
+          <t>Proximal Methods</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2543,24 +2543,24 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>665</v>
+        <v>965</v>
       </c>
       <c r="E29" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2577,38 +2577,38 @@
         <v>7</v>
       </c>
       <c r="L29" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M29" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="N29" t="n">
-        <v>281</v>
+        <v>312</v>
       </c>
       <c r="O29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q29" t="n">
         <v>0</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>The Pinball Loss and the Population Quantile, Linear Quantile Regression, The LP Reformulation, Equivariance Under Monotone Transformations, Asymptotic Theory: Koenker–Bassett 1978, Knight 1998, Multi-Quantile Estimation, Crossing, and Rearrangement, Penalized Quantile Regression, Quantile Regression as the Base Learner of Conformalized QR, Connections and Further Reading</t>
+          <t>Overview &amp; Motivation, The Proximal Operator, Proximal Operator Catalog, The Moreau Envelope, Proximal Gradient Descent, ISTA &amp; Soft-Thresholding, FISTA: Accelerated Proximal Gradient, Douglas–Rachford Splitting, ADMM, Convergence Analysis, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>graph-theory</t>
+          <t>nonparametric-ml</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Random Walks &amp; Mixing</t>
+          <t>Quantile Regression</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2617,24 +2617,24 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1500</v>
+        <v>665</v>
       </c>
       <c r="E30" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2648,41 +2648,41 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L30" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="M30" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="N30" t="n">
-        <v>208</v>
+        <v>281</v>
       </c>
       <c r="O30" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P30" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q30" t="n">
         <v>0</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, 1. Markov Chains on Graphs, 2. Stationary Distribution &amp; Convergence, 3. Total Variation &amp; Mixing Time, 4. Spectral Analysis of Mixing, 5. Lazy Random Walks, 6. Hitting Times &amp; Commute Times, 7. Effective Resistance &amp; Electrical Networks, 8. Applications: PageRank, DeepWalk, Label Propagation, 9. Computational Notes, 10. Connections &amp; Further Reading</t>
+          <t>The Pinball Loss and the Population Quantile, Linear Quantile Regression, The LP Reformulation, Equivariance Under Monotone Transformations, Asymptotic Theory: Koenker–Bassett 1978, Knight 1998, Multi-Quantile Estimation, Crossing, and Rearrangement, Penalized Quantile Regression, Quantile Regression as the Base Learner of Conformalized QR, Connections and Further Reading</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nonparametric-ml</t>
+          <t>graph-theory</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Rank Tests &amp; Permutation Inference</t>
+          <t>Random Walks &amp; Mixing</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2691,14 +2691,14 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1879</v>
+        <v>1500</v>
       </c>
       <c r="E31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2722,41 +2722,41 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L31" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="M31" t="n">
-        <v>68</v>
+        <v>23</v>
       </c>
       <c r="N31" t="n">
-        <v>661</v>
+        <v>208</v>
       </c>
       <c r="O31" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="P31" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="Q31" t="n">
         <v>0</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>From the Sign Test to Wilcoxon Signed-Rank, The Permutation Principle and Exchangeability, Wilcoxon Rank-Sum and Mann-Whitney $U$, Kruskal-Wallis: The $k$-Sample Extension, Asymptotic Relative Efficiency (Pitman), The Hodges-Lehmann Estimator, Permutation Tests with Non-Rank Statistics, Limitations: Ties, Power, and the Covariate Problem, Notation Reference, Connections and Further Reading</t>
+          <t>Overview &amp; Motivation, 1. Markov Chains on Graphs, 2. Stationary Distribution &amp; Convergence, 3. Total Variation &amp; Mixing Time, 4. Spectral Analysis of Mixing, 5. Lazy Random Walks, 6. Hitting Times &amp; Commute Times, 7. Effective Resistance &amp; Electrical Networks, 8. Applications: PageRank, DeepWalk, Label Propagation, 9. Computational Notes, 10. Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>information-theory</t>
+          <t>nonparametric-ml</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Rate-Distortion Theory</t>
+          <t>Rank Tests &amp; Permutation Inference</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2765,14 +2765,14 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>826</v>
+        <v>1879</v>
       </c>
       <c r="E32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2796,53 +2796,53 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="M32" t="n">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="N32" t="n">
-        <v>264</v>
+        <v>661</v>
       </c>
       <c r="O32" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="P32" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="Q32" t="n">
         <v>0</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Distortion Measures, The Rate-Distortion Function, The Rate-Distortion Theorem, Closed-Form Solutions, The Blahut–Arimoto Algorithm, The Information Bottleneck, Computational Notes, Connections &amp; Further Reading</t>
+          <t>From the Sign Test to Wilcoxon Signed-Rank, The Permutation Principle and Exchangeability, Wilcoxon Rank-Sum and Mann-Whitney $U$, Kruskal-Wallis: The $k$-Sample Extension, Asymptotic Relative Efficiency (Pitman), The Hodges-Lehmann Estimator, Permutation Tests with Non-Rank Statistics, Limitations: Ties, Power, and the Covariate Problem, Notation Reference, Connections and Further Reading</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>geometry</t>
+          <t>information-theory</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Riemannian Geometry</t>
+          <t>Rate-Distortion Theory</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2058</v>
+        <v>826</v>
       </c>
       <c r="E33" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -2870,16 +2870,16 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L33" t="n">
+        <v>25</v>
+      </c>
+      <c r="M33" t="n">
         <v>28</v>
       </c>
-      <c r="M33" t="n">
-        <v>37</v>
-      </c>
       <c r="N33" t="n">
-        <v>356</v>
+        <v>264</v>
       </c>
       <c r="O33" t="n">
         <v>6</v>
@@ -2892,31 +2892,31 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Riemannian Metrics, Lengths of Curves and Riemannian Distance, Musical Isomorphisms, The Levi-Civita Connection, Parallel Transport, Riemannian Volume Form and Integration, Isometries and Killing Vector Fields, Computational Notes, Connections to Machine Learning, Connections and Further Reading</t>
+          <t>Overview &amp; Motivation, Distortion Measures, The Rate-Distortion Function, The Rate-Distortion Theorem, Closed-Form Solutions, The Blahut–Arimoto Algorithm, The Information Bottleneck, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>information-theory</t>
+          <t>geometry</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Shannon Entropy &amp; Mutual Information</t>
+          <t>Riemannian Geometry</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>foundational</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1643</v>
+        <v>2058</v>
       </c>
       <c r="E34" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -2944,16 +2944,16 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L34" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="M34" t="n">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="N34" t="n">
-        <v>210</v>
+        <v>356</v>
       </c>
       <c r="O34" t="n">
         <v>6</v>
@@ -2966,31 +2966,31 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Information Content &amp; Shannon Entropy, Joint Entropy &amp; Conditional Entropy, Mutual Information, The Data Processing Inequality, Differential Entropy, Source Coding &amp; Compression, Entropy Rate, Computational Notes, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, Riemannian Metrics, Lengths of Curves and Riemannian Distance, Musical Isomorphisms, The Levi-Civita Connection, Parallel Transport, Riemannian Volume Form and Integration, Isometries and Killing Vector Fields, Computational Notes, Connections to Machine Learning, Connections and Further Reading</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>topology</t>
+          <t>information-theory</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Sheaf Theory</t>
+          <t>Shannon Entropy &amp; Mutual Information</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>foundational</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>3569</v>
+        <v>1643</v>
       </c>
       <c r="E35" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3018,16 +3018,16 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L35" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="M35" t="n">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="N35" t="n">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="O35" t="n">
         <v>6</v>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Presheaves and Sheaves, Cellular Sheaves on Graphs, Sheaf Cohomology, The Sheaf Laplacian, Cosheaves and Duality, Applications, The Topology &amp; TDA Track: A Capstone View, Exercises</t>
+          <t>Overview &amp; Motivation, Information Content &amp; Shannon Entropy, Joint Entropy &amp; Conditional Entropy, Mutual Information, The Data Processing Inequality, Differential Entropy, Source Coding &amp; Compression, Entropy Rate, Computational Notes, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
@@ -3052,19 +3052,19 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Simplicial Complexes</t>
+          <t>Sheaf Theory</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>foundational</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>648</v>
+        <v>3569</v>
       </c>
       <c r="E36" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -3073,12 +3073,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3092,53 +3092,53 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L36" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="M36" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="N36" t="n">
-        <v>240</v>
+        <v>214</v>
       </c>
       <c r="O36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q36" t="n">
         <v>0</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Formal Framework, Homology Preview, The Euler Characteristic, Other Complex Constructions, Computational Notes, Visual Intuition, Working Code, Connections &amp; Cross-Track Bridges, Exercises</t>
+          <t>Overview &amp; Motivation, Presheaves and Sheaves, Cellular Sheaves on Graphs, Sheaf Cohomology, The Sheaf Laplacian, Cosheaves and Duality, Applications, The Topology &amp; TDA Track: A Capstone View, Exercises</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>geometry</t>
+          <t>topology</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Smooth Manifolds</t>
+          <t>Simplicial Complexes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>foundational</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4886</v>
+        <v>648</v>
       </c>
       <c r="E37" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3169,50 +3169,50 @@
         <v>5</v>
       </c>
       <c r="L37" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="M37" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="N37" t="n">
-        <v>375</v>
+        <v>240</v>
       </c>
       <c r="O37" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P37" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q37" t="n">
         <v>0</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Topological Manifolds, Charts and Atlases, Smooth Manifolds, A Gallery of Smooth Manifolds, Smooth Maps &amp; Diffeomorphisms, Tangent Vectors &amp; Tangent Spaces, The Differential (Pushforward), Partitions of Unity, Computational Notes, The Whitney Embedding Theorem &amp; Connections</t>
+          <t>Overview &amp; Motivation, Formal Framework, Homology Preview, The Euler Characteristic, Other Complex Constructions, Computational Notes, Visual Intuition, Working Code, Connections &amp; Cross-Track Bridges, Exercises</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>linear-algebra</t>
+          <t>geometry</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>The Spectral Theorem</t>
+          <t>Smooth Manifolds</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>foundational</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1604</v>
+        <v>4886</v>
       </c>
       <c r="E38" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3243,47 +3243,47 @@
         <v>5</v>
       </c>
       <c r="L38" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="M38" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="N38" t="n">
-        <v>226</v>
+        <v>375</v>
       </c>
       <c r="O38" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P38" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q38" t="n">
         <v>0</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, Eigenvalues &amp; Eigenvectors, Symmetric Matrices &amp; Orthogonality, The Spectral Theorem, The Rayleigh Quotient, Quadratic Forms &amp; Definiteness, Spectral Decomposition in Practice, Application: Spectral Clustering, Application: PCA Preview, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, Topological Manifolds, Charts and Atlases, Smooth Manifolds, A Gallery of Smooth Manifolds, Smooth Maps &amp; Diffeomorphisms, Tangent Vectors &amp; Tangent Spaces, The Differential (Pushforward), Partitions of Unity, Computational Notes, The Whitney Embedding Theorem &amp; Connections</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>topology</t>
+          <t>linear-algebra</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Statistical TDA</t>
+          <t>The Spectral Theorem</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>foundational</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3177</v>
+        <v>1604</v>
       </c>
       <c r="E39" t="n">
         <v>10</v>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3314,50 +3314,50 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L39" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="M39" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="N39" t="n">
-        <v>201</v>
+        <v>226</v>
       </c>
       <c r="O39" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P39" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q39" t="n">
         <v>0</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, 1. Stability &amp; Convergence, 2. Confidence Sets for Persistence Diagrams, 3. Persistence Landscapes &amp; Images, 4. Hypothesis Testing, 5. Application: Financial Market Regimes, Summary, Working Code, Connections &amp; Cross-Track Bridges, Exercises</t>
+          <t>Overview &amp; Motivation, Eigenvalues &amp; Eigenvectors, Symmetric Matrices &amp; Orthogonality, The Spectral Theorem, The Rayleigh Quotient, Quadratic Forms &amp; Definiteness, Spectral Decomposition in Practice, Application: Spectral Clustering, Application: PCA Preview, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>linear-algebra</t>
+          <t>topology</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Singular Value Decomposition</t>
+          <t>Statistical TDA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2694</v>
+        <v>3177</v>
       </c>
       <c r="E40" t="n">
         <v>10</v>
@@ -3374,7 +3374,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3388,29 +3388,29 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L40" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="M40" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N40" t="n">
-        <v>228</v>
+        <v>201</v>
       </c>
       <c r="O40" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P40" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q40" t="n">
         <v>0</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, From the Spectral Theorem to the SVD, The SVD: Statement and Proof, Geometric Interpretation, Low-Rank Approximation, Computing the SVD in Practice, Application: Image Compression, Application: Latent Semantic Analysis, The SVD–PCA Connection, Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, 1. Stability &amp; Convergence, 2. Confidence Sets for Persistence Diagrams, 3. Persistence Landscapes &amp; Images, 4. Hypothesis Testing, 5. Application: Financial Market Regimes, Summary, Working Code, Connections &amp; Cross-Track Bridges, Exercises</t>
         </is>
       </c>
     </row>
@@ -3422,19 +3422,19 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Tensor Decompositions</t>
+          <t>Singular Value Decomposition</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>3613</v>
+        <v>2694</v>
       </c>
       <c r="E41" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3462,41 +3462,41 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L41" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="M41" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N41" t="n">
-        <v>245</v>
+        <v>228</v>
       </c>
       <c r="O41" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P41" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q41" t="n">
         <v>0</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, 1. Tensor Fundamentals, 2. CP Decomposition (CANDECOMP/PARAFAC), 3. Tucker Decomposition, 4. Higher-Order SVD (HOSVD), 5. Tensor Train Decomposition, 6. The t-SVD (Tensor SVD via the Fourier Domain), 7. Multilinear PCA, 8. Applications, 9. Computational Notes, 10. Connections &amp; Further Reading</t>
+          <t>Overview &amp; Motivation, From the Spectral Theorem to the SVD, The SVD: Statement and Proof, Geometric Interpretation, Low-Rank Approximation, Computing the SVD in Practice, Application: Image Compression, Application: Latent Semantic Analysis, The SVD–PCA Connection, Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>nonparametric-ml</t>
+          <t>linear-algebra</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Statistical Depth</t>
+          <t>Tensor Decompositions</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3505,10 +3505,10 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>4158</v>
+        <v>3613</v>
       </c>
       <c r="E42" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3536,50 +3536,50 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L42" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="M42" t="n">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="N42" t="n">
-        <v>193</v>
+        <v>245</v>
       </c>
       <c r="O42" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="P42" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="Q42" t="n">
         <v>0</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Overview, 1. From quantile to depth, 2. Tukey halfspace depth, 3. A zoo of depth functions, 4. Theory and computation, 5. ML applications, 6. Connections and limits</t>
+          <t>Overview &amp; Motivation, 1. Tensor Fundamentals, 2. CP Decomposition (CANDECOMP/PARAFAC), 3. Tucker Decomposition, 4. Higher-Order SVD (HOSVD), 5. Tensor Train Decomposition, 6. The t-SVD (Tensor SVD via the Fourier Domain), 7. Multilinear PCA, 8. Applications, 9. Computational Notes, 10. Connections &amp; Further Reading</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>bayesian-ml</t>
+          <t>nonparametric-ml</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Variational Inference</t>
+          <t>Statistical Depth</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>8739</v>
+        <v>4158</v>
       </c>
       <c r="E43" t="n">
         <v>7</v>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3613,26 +3613,26 @@
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="M43" t="n">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="N43" t="n">
-        <v>567</v>
+        <v>193</v>
       </c>
       <c r="O43" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="P43" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="Q43" t="n">
         <v>0</v>
       </c>
-      <c r="R43" s="2" t="inlineStr">
-        <is>
-          <t>Overview, 1. The intractable posterior, 2. The ELBO, 3. Mean-field VI and CAVI, 4. Stochastic and black-box VI, 5. Beyond mean-field: structured VI and normalizing flows, 6. Connections and limits</t>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Overview, 1. From quantile to depth, 2. Tukey halfspace depth, 3. A zoo of depth functions, 4. Theory and computation, 5. ML applications, 6. Connections and limits</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Gaussian Processes</t>
+          <t>Variational Inference</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3653,7 +3653,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2764</v>
+        <v>8739</v>
       </c>
       <c r="E44" t="n">
         <v>7</v>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -3690,23 +3690,23 @@
         <v>15</v>
       </c>
       <c r="M44" t="n">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="N44" t="n">
-        <v>517</v>
+        <v>567</v>
       </c>
       <c r="O44" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="P44" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="Q44" t="n">
         <v>0</v>
       </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>Overview, 1. From parametric Bayes to function-space priors, 2. Gaussian processes as priors over functions, 3. Conjugate GP regression, 4. Kernel design and the inductive bias, 5. Learning hyperparameters from the marginal likelihood, 6. Scaling, neighbors, and limits</t>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>Overview, 1. The intractable posterior, 2. The ELBO, 3. Mean-field VI and CAVI, 4. Stochastic and black-box VI, 5. Beyond mean-field: structured VI and normalizing flows, 6. Connections and limits</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Probabilistic Programming</t>
+          <t>Gaussian Processes</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>9437</v>
+        <v>2764</v>
       </c>
       <c r="E45" t="n">
         <v>7</v>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -3758,29 +3758,29 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="M45" t="n">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="N45" t="n">
-        <v>266</v>
+        <v>517</v>
       </c>
       <c r="O45" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="P45" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="Q45" t="n">
         <v>0</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Overview, 1. From explicit Bayes to declarative Bayes, 2. Anatomy of a probabilistic program, 3. Constrained-to-unconstrained transforms, 4. Inference dispatch: NUTS, ADVI, and MAP, 5. The Bayesian workflow on eight schools, 6. Limits, alternatives, and connections</t>
+          <t>Overview, 1. From parametric Bayes to function-space priors, 2. Gaussian processes as priors over functions, 3. Conjugate GP regression, 4. Kernel design and the inductive bias, 5. Learning hyperparameters from the marginal likelihood, 6. Scaling, neighbors, and limits</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Mixed-Effects Models</t>
+          <t>Probabilistic Programming</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3801,7 +3801,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>8644</v>
+        <v>9437</v>
       </c>
       <c r="E46" t="n">
         <v>7</v>
@@ -3832,16 +3832,16 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L46" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="M46" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="N46" t="n">
-        <v>616</v>
+        <v>266</v>
       </c>
       <c r="O46" t="n">
         <v>18</v>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Overview, 1. Three responses to grouped data, 2. The linear mixed model, 3. Henderson's mixed-model equations and BLUP, 4. REML for variance components, 5. The frequentist–Bayesian bridge, 6. Connections, limits, and references</t>
+          <t>Overview, 1. From explicit Bayes to declarative Bayes, 2. Anatomy of a probabilistic program, 3. Constrained-to-unconstrained transforms, 4. Inference dispatch: NUTS, ADVI, and MAP, 5. The Bayesian workflow on eight schools, 6. Limits, alternatives, and connections</t>
         </is>
       </c>
     </row>
@@ -3866,19 +3866,19 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bayesian Neural Networks</t>
+          <t>Mixed-Effects Models</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>11882</v>
+        <v>8644</v>
       </c>
       <c r="E47" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3906,29 +3906,29 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L47" t="n">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="M47" t="n">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="N47" t="n">
-        <v>730</v>
+        <v>616</v>
       </c>
       <c r="O47" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="P47" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="Q47" t="n">
         <v>0</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>Overview, 1. Why Bayesian over the weights, 2. The weight-space posterior, 3. The Laplace approximation, 4. MC-dropout as approximate variational inference, 5. Deep ensembles as a function-space posterior proxy, 6. Stochastic-gradient Langevin dynamics (SGLD), 7. Stochastic-gradient HMC (SGHMC), 8. Calibration and uncertainty quantification, 9. Function-space view: NNGP, NTK, and open problems, Connections and further reading</t>
+          <t>Overview, 1. Three responses to grouped data, 2. The linear mixed model, 3. Henderson's mixed-model equations and BLUP, 4. REML for variance components, 5. The frequentist–Bayesian bridge, 6. Connections, limits, and references</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Variational Bayes for Model Selection</t>
+          <t>Bayesian Neural Networks</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3949,10 +3949,10 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>8894</v>
+        <v>11882</v>
       </c>
       <c r="E48" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3980,53 +3980,53 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L48" t="n">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="M48" t="n">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="N48" t="n">
-        <v>194</v>
+        <v>730</v>
       </c>
       <c r="O48" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P48" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q48" t="n">
         <v>0</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Overview &amp; Motivation, From ELBO to log-evidence — the VBMS criterion, Laplace approximation and the BIC bridge, Variational Bayes for Bayesian GMMs, Comparing Bayesian regression models (polynomial Bayes factors), The KL projection bias, Asymmetric bias and ranking preservation, Importance-weighted ELBO and bias correction, Annealed importance sampling as the gold-standard reference, The MDL connection — variational free energy as bits-back coding, Computational notes, VBMS in modern ML, Connections and limits</t>
+          <t>Overview, 1. Why Bayesian over the weights, 2. The weight-space posterior, 3. The Laplace approximation, 4. MC-dropout as approximate variational inference, 5. Deep ensembles as a function-space posterior proxy, 6. Stochastic-gradient Langevin dynamics (SGLD), 7. Stochastic-gradient HMC (SGHMC), 8. Calibration and uncertainty quantification, 9. Function-space view: NNGP, NTK, and open problems, Connections and further reading</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>supervised-learning</t>
+          <t>bayesian-ml</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Kernel Regression</t>
+          <t>Variational Bayes for Model Selection</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>7098</v>
+        <v>8894</v>
       </c>
       <c r="E49" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -4054,29 +4054,29 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="M49" t="n">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="N49" t="n">
-        <v>634</v>
+        <v>194</v>
       </c>
       <c r="O49" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="P49" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="Q49" t="n">
         <v>0</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1. From parametric to nonparametric: the local-averaging idea | 2. The Nadaraya–Watson estimator | 3. Pointwise bias at an interior point | 4. Pointwise variance and the AMISE | 5. Bandwidth selection in practice | 6. Multivariate regression and the curse of dimensionality | 7. Kernel choice: what matters and what doesn't | 8. Boundary bias and the local-linear fix | 9. Connections and applications | Connections and Further Reading</t>
+          <t>Overview &amp; Motivation, From ELBO to log-evidence — the VBMS criterion, Laplace approximation and the BIC bridge, Variational Bayes for Bayesian GMMs, Comparing Bayesian regression models (polynomial Bayes factors), The KL projection bias, Asymmetric bias and ranking preservation, Importance-weighted ELBO and bias correction, Annealed importance sampling as the gold-standard reference, The MDL connection — variational free energy as bits-back coding, Computational notes, VBMS in modern ML, Connections and limits</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Local Polynomial Regression</t>
+          <t>Kernel Regression</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -4097,10 +4097,10 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6856</v>
+        <v>7098</v>
       </c>
       <c r="E50" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -4128,29 +4128,29 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L50" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="M50" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="N50" t="n">
-        <v>852</v>
+        <v>634</v>
       </c>
       <c r="O50" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="P50" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="Q50" t="n">
         <v>0</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>1. From local-linear to degree-$p$ | 2. The degree-$p$ local polynomial estimator | 3. The equivalent-kernel formulation | 4. Bias and variance at general $p$ | 5. The boundary and the odd-vs-even degree story | 6. Boundary behavior across the full support | 7. Bandwidth selection at general $p$ | 8. Multivariate local polynomials | 9. Derivative estimation | 10. Connections to smoothing splines | 11. Connections to additive models | 12. Connections, applications, and limits | Connections and Further Reading</t>
+          <t>1. From parametric to nonparametric: the local-averaging idea | 2. The Nadaraya–Watson estimator | 3. Pointwise bias at an interior point | 4. Pointwise variance and the AMISE | 5. Bandwidth selection in practice | 6. Multivariate regression and the curse of dimensionality | 7. Kernel choice: what matters and what doesn't | 8. Boundary bias and the local-linear fix | 9. Connections and applications | Connections and Further Reading</t>
         </is>
       </c>
     </row>
@@ -4162,19 +4162,19 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>High-Dimensional Regression</t>
+          <t>Local Polynomial Regression</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>17945</v>
+        <v>6856</v>
       </c>
       <c r="E51" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -4202,41 +4202,41 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="M51" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="N51" t="n">
-        <v>229</v>
+        <v>852</v>
       </c>
       <c r="O51" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="P51" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="Q51" t="n">
         <v>0</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>1. From OLS to penalized regression | 2. The lasso estimator | 3. Solving the lasso | 4. Bias-variance for the lasso | 5. The lasso oracle inequality | 6. Variable-selection consistency | 7. Cross-validation for λ | 8. Ridge, elastic net, and adaptive lasso | 9. Geometry of the high-dimensional regime | 10. Post-selection inference and the debiased lasso | 11. Generalized lasso for non-Gaussian responses | 12. Connections, applications, and limits</t>
+          <t>1. From local-linear to degree-$p$ | 2. The degree-$p$ local polynomial estimator | 3. The equivalent-kernel formulation | 4. Bias and variance at general $p$ | 5. The boundary and the odd-vs-even degree story | 6. Boundary behavior across the full support | 7. Bandwidth selection at general $p$ | 8. Multivariate local polynomials | 9. Derivative estimation | 10. Connections to smoothing splines | 11. Connections to additive models | 12. Connections, applications, and limits | Connections and Further Reading</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>unsupervised</t>
+          <t>supervised-learning</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Normalizing Flows</t>
+          <t>High-Dimensional Regression</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -4245,7 +4245,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>14049</v>
+        <v>17945</v>
       </c>
       <c r="E52" t="n">
         <v>12</v>
@@ -4276,53 +4276,53 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L52" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="M52" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="N52" t="n">
-        <v>757</v>
+        <v>229</v>
       </c>
       <c r="O52" t="n">
-        <v>23</v>
+        <v>50</v>
       </c>
       <c r="P52" t="n">
-        <v>23</v>
+        <v>50</v>
       </c>
       <c r="Q52" t="n">
         <v>0</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Motivation: explicit-density generative models, Change of variables in d dimensions, The normalizing-flow framework, Coupling layers — NICE and RealNVP, Autoregressive flows — MAF and IAF, Multi-scale and image-domain architectures, Maximum-likelihood training, Expressivity and universality, Flows for variational inference, Flows for density estimation, Worked example: 2-moons end-to-end, Connections, applications, and limits</t>
+          <t>1. From OLS to penalized regression | 2. The lasso estimator | 3. Solving the lasso | 4. Bias-variance for the lasso | 5. The lasso oracle inequality | 6. Variable-selection consistency | 7. Cross-validation for λ | 8. Ridge, elastic net, and adaptive lasso | 9. Geometry of the high-dimensional regime | 10. Post-selection inference and the debiased lasso | 11. Generalized lasso for non-Gaussian responses | 12. Connections, applications, and limits</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>learning-theory</t>
+          <t>unsupervised</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Generalization Bounds</t>
+          <t>Normalizing Flows</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>13112</v>
+        <v>14049</v>
       </c>
       <c r="E53" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4350,29 +4350,29 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" t="n">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="M53" t="n">
         <v>68</v>
       </c>
       <c r="N53" t="n">
-        <v>875</v>
+        <v>757</v>
       </c>
       <c r="O53" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="P53" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="Q53" t="n">
         <v>0</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Motivation: why bound the generalization gap?, The generalization gap and its decomposition, Finite-class warmup, Uniform convergence and Glivenko–Cantelli, Rademacher complexity, Symmetrization, McDiarmid + Rademacher → uniform convergence, Real-valued function classes, Data-dependent bounds, Margin bounds, Algorithmic stability bounds, Worked example: empirical Rademacher and vacuousness, Computational notes, Connections and limits</t>
+          <t>Motivation: explicit-density generative models, Change of variables in d dimensions, The normalizing-flow framework, Coupling layers — NICE and RealNVP, Autoregressive flows — MAF and IAF, Multi-scale and image-domain architectures, Maximum-likelihood training, Expressivity and universality, Flows for variational inference, Flows for density estimation, Worked example: 2-moons end-to-end, Connections, applications, and limits</t>
         </is>
       </c>
     </row>
@@ -4384,16 +4384,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PAC-Bayes Bounds</t>
+          <t>Generalization Bounds</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>8107</v>
+        <v>13112</v>
       </c>
       <c r="E54" t="n">
         <v>14</v>
@@ -4410,7 +4410,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -4424,29 +4424,29 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="M54" t="n">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="N54" t="n">
-        <v>763</v>
+        <v>875</v>
       </c>
       <c r="O54" t="n">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="P54" t="n">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="Q54" t="n">
         <v>0</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Motivation: beyond uniform convergence, The PAC-Bayes setup, The change-of-measure inequality, The McAllester bound, The Seeger / kl-form bound, The Catoni / linear bound and the Gibbs posterior, Refinements, Choosing prior and posterior in continuous classes, The Bayesian–PAC-Bayes correspondence, Three bounds on the running example, Non-vacuous deep-network bounds (Dziugaite–Roy 2017), ML applications, Computational notes, Connections and limits</t>
+          <t>Motivation: why bound the generalization gap?, The generalization gap and its decomposition, Finite-class warmup, Uniform convergence and Glivenko–Cantelli, Rademacher complexity, Symmetrization, McDiarmid + Rademacher → uniform convergence, Real-valued function classes, Data-dependent bounds, Margin bounds, Algorithmic stability bounds, Worked example: empirical Rademacher and vacuousness, Computational notes, Connections and limits</t>
         </is>
       </c>
     </row>
@@ -4458,16 +4458,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Structural Risk Minimization</t>
+          <t>PAC-Bayes Bounds</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>8770</v>
+        <v>8107</v>
       </c>
       <c r="E55" t="n">
         <v>14</v>
@@ -4501,26 +4501,26 @@
         <v>1</v>
       </c>
       <c r="L55" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="M55" t="n">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="N55" t="n">
-        <v>737</v>
+        <v>763</v>
       </c>
       <c r="O55" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="P55" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="Q55" t="n">
         <v>0</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Motivation: why capacity control matters; The nested-family setup; The SRM principle; Classical VC-bound SRM (Vapnik 1995/1998); Rademacher-complexity SRM (Bartlett-Mendelson 2002); Penalized ERM and soft SRM; SRM as regularization; SRM and information criteria; SRM and PAC-Bayes; Cross-validation as data-driven SRM; Worked example: polynomial regression with SRM; SRM in practice: SVMs and beyond; Connections and limits; Computational notes</t>
+          <t>Motivation: beyond uniform convergence, The PAC-Bayes setup, The change-of-measure inequality, The McAllester bound, The Seeger / kl-form bound, The Catoni / linear bound and the Gibbs posterior, Refinements, Choosing prior and posterior in continuous classes, The Bayesian–PAC-Bayes correspondence, Three bounds on the running example, Non-vacuous deep-network bounds (Dziugaite–Roy 2017), ML applications, Computational notes, Connections and limits</t>
         </is>
       </c>
     </row>
@@ -4532,16 +4532,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Causal Inference Methods</t>
+          <t>Structural Risk Minimization</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>4790</v>
+        <v>8770</v>
       </c>
       <c r="E56" t="n">
         <v>14</v>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4572,29 +4572,29 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M56" t="n">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="N56" t="n">
-        <v>347</v>
+        <v>737</v>
       </c>
       <c r="O56" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="P56" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="Q56" t="n">
         <v>0</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>§1 Motivation: prediction is not enough, §2 The potential-outcomes framework, §3 Identification under ignorability and positivity, §4 The IPW estimator, §5 Outcome regression and the g-formula, §6 Augmented IPW and double robustness, §7 Targeted Maximum Likelihood (TMLE), §8 Double / debiased Machine Learning (DML), §9 Instrumental variables, §10 Front-door identification, §11 Heterogeneous treatment effects, §12 Sensitivity analysis, §13 Worked example: end-to-end on the Robinson DGP, §14 Connections and limits</t>
+          <t>Motivation: why capacity control matters; The nested-family setup; The SRM principle; Classical VC-bound SRM (Vapnik 1995/1998); Rademacher-complexity SRM (Bartlett-Mendelson 2002); Penalized ERM and soft SRM; SRM as regularization; SRM and information criteria; SRM and PAC-Bayes; Cross-validation as data-driven SRM; Worked example: polynomial regression with SRM; SRM in practice: SVMs and beyond; Connections and limits; Computational notes</t>
         </is>
       </c>
     </row>
@@ -4606,19 +4606,19 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VC Dimension</t>
+          <t>Causal Inference Methods</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>4837</v>
+        <v>4790</v>
       </c>
       <c r="E57" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -4649,26 +4649,26 @@
         <v>0</v>
       </c>
       <c r="L57" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="M57" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="N57" t="n">
-        <v>701</v>
+        <v>347</v>
       </c>
       <c r="O57" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="P57" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="Q57" t="n">
         <v>0</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Motivation: why finite-class arguments break for infinite hypothesis classes, Shattering: the combinatorial substitute for |H|, The growth function Π(n), The VC dimension, The Sauer–Shelah lemma, The Fundamental Theorem of Statistical Learning, Realizable versus agnostic rates, VC dimension of canonical classes, From VC dimension to Rademacher complexity, Integrative worked example: half-planes and rectangles, end to end, ML applications, Computational notes, Connections and limits</t>
+          <t>§1 Motivation: prediction is not enough, §2 The potential-outcomes framework, §3 Identification under ignorability and positivity, §4 The IPW estimator, §5 Outcome regression and the g-formula, §6 Augmented IPW and double robustness, §7 Targeted Maximum Likelihood (TMLE), §8 Double / debiased Machine Learning (DML), §9 Instrumental variables, §10 Front-door identification, §11 Heterogeneous treatment effects, §12 Sensitivity analysis, §13 Worked example: end-to-end on the Robinson DGP, §14 Connections and limits</t>
         </is>
       </c>
     </row>
@@ -4680,19 +4680,19 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Double Descent</t>
+          <t>VC Dimension</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>11756</v>
+        <v>4837</v>
       </c>
       <c r="E58" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -4706,7 +4706,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4720,29 +4720,29 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L58" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="M58" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="N58" t="n">
-        <v>953</v>
+        <v>701</v>
       </c>
       <c r="O58" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="P58" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="Q58" t="n">
         <v>0</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Motivation: the empirical phenomenon, The classical story being revised, The interpolation threshold, Beyond the threshold: ridgeless regression, Random matrix theory bridge: Marchenko–Pastur, Asymptotic bias-variance under ridgeless OLS, Sample-wise vs model-wise double descent, Random features and the kernel limit, Implicit regularization, Deep double descent (sidebar), Effective dimension, Connections to PAC-Bayes and SRM, Computational notes, Connections and limits</t>
+          <t>Motivation: why finite-class arguments break for infinite hypothesis classes, Shattering: the combinatorial substitute for |H|, The growth function Π(n), The VC dimension, The Sauer–Shelah lemma, The Fundamental Theorem of Statistical Learning, Realizable versus agnostic rates, VC dimension of canonical classes, From VC dimension to Rademacher complexity, Integrative worked example: half-planes and rectangles, end to end, ML applications, Computational notes, Connections and limits</t>
         </is>
       </c>
     </row>
@@ -4754,16 +4754,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Uncertainty Quantification</t>
+          <t>Double Descent</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>intermediate</t>
+          <t>advanced</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>4419</v>
+        <v>11756</v>
       </c>
       <c r="E59" t="n">
         <v>14</v>
@@ -4780,7 +4780,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4794,29 +4794,29 @@
         </is>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L59" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="M59" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="N59" t="n">
-        <v>180</v>
+        <v>953</v>
       </c>
       <c r="O59" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="P59" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="Q59" t="n">
         <v>0</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Motivation: why claimed uncertainty often fails to match empirical uncertainty; Aleatoric vs epistemic decomposition; Calibration; Proper scoring rules; Predictive intervals across paradigms; Bootstrap-based UQ; Bayesian UQ in NumPy; Conformal UQ; Deep-ensemble UQ; UQ in the over-parameterized regime; Evaluating UQ at distribution shift; Decision-theoretic UQ; Computational notes; Connections and limits</t>
+          <t>Motivation: the empirical phenomenon, The classical story being revised, The interpolation threshold, Beyond the threshold: ridgeless regression, Random matrix theory bridge: Marchenko–Pastur, Asymptotic bias-variance under ridgeless OLS, Sample-wise vs model-wise double descent, Random features and the kernel limit, Implicit regularization, Deep double descent (sidebar), Effective dimension, Connections to PAC-Bayes and SRM, Computational notes, Connections and limits</t>
         </is>
       </c>
     </row>
@@ -4828,23 +4828,23 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Semiparametric Inference</t>
+          <t>Uncertainty Quantification</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>advanced</t>
+          <t>intermediate</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>9141</v>
+        <v>4419</v>
       </c>
       <c r="E60" t="n">
         <v>14</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4871,98 +4871,172 @@
         <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="M60" t="n">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="N60" t="n">
-        <v>615</v>
+        <v>180</v>
       </c>
       <c r="O60" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="P60" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="Q60" t="n">
         <v>0</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Motivation, Tangent spaces, Efficient influence functions, Semiparametric efficiency bound, One-step estimators, Targeted maximum likelihood (TMLE), Double / debiased machine learning (DML), Sample-splitting and cross-fitting, Worked examples, Inference and confidence intervals, Connections to uncertainty quantification, Connections to causal inference, Computational notes, Connections and limits</t>
+          <t>Motivation: why claimed uncertainty often fails to match empirical uncertainty; Aleatoric vs epistemic decomposition; Calibration; Proper scoring rules; Predictive intervals across paradigms; Bootstrap-based UQ; Bayesian UQ in NumPy; Conformal UQ; Deep-ensemble UQ; UQ in the over-parameterized regime; Evaluating UQ at distribution shift; Decision-theoretic UQ; Computational notes; Connections and limits</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>learning-theory</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Semiparametric Inference</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>9141</v>
+      </c>
+      <c r="E61" t="n">
+        <v>14</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="n">
+        <v>13</v>
+      </c>
+      <c r="M61" t="n">
+        <v>52</v>
+      </c>
+      <c r="N61" t="n">
+        <v>615</v>
+      </c>
+      <c r="O61" t="n">
+        <v>16</v>
+      </c>
+      <c r="P61" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Motivation, Tangent spaces, Efficient influence functions, Semiparametric efficiency bound, One-step estimators, Targeted maximum likelihood (TMLE), Double / debiased machine learning (DML), Sample-splitting and cross-fitting, Worked examples, Inference and confidence intervals, Connections to uncertainty quantification, Connections to causal inference, Computational notes, Connections and limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>unsupervised</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>Clustering</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>intermediate</t>
         </is>
       </c>
-      <c r="D61" t="n">
+      <c r="D62" t="n">
         <v>6346</v>
       </c>
-      <c r="E61" t="n">
+      <c r="E62" t="n">
         <v>12</v>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K61" t="n">
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K62" t="n">
         <v>1</v>
       </c>
-      <c r="L61" t="n">
+      <c r="L62" t="n">
         <v>20</v>
       </c>
-      <c r="M61" t="n">
+      <c r="M62" t="n">
         <v>37</v>
       </c>
-      <c r="N61" t="n">
+      <c r="N62" t="n">
         <v>524</v>
       </c>
-      <c r="O61" t="n">
+      <c r="O62" t="n">
         <v>41</v>
       </c>
-      <c r="P61" t="n">
+      <c r="P62" t="n">
         <v>41</v>
       </c>
-      <c r="Q61" t="n">
-        <v>0</v>
-      </c>
-      <c r="R61" t="inlineStr">
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" t="inlineStr">
         <is>
           <t>Motivation: when linear partitions fail, The KDE substrate and the mode-finding picture, Mean-shift as gradient ascent on f_h, Convergence theory, Bandwidth resolution and the mode tree, Kernel-function choice, From trajectories to clusters, Practical mean-shift, k-means as the h-to-0 Voronoi limit, GMM-via-EM and soft assignment, Pointers: spectral and density-based clustering, Connections limits and forward pointers</t>
         </is>
@@ -5414,10 +5488,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C11" t="n">
-        <v>8393</v>
+        <v>8724</v>
       </c>
       <c r="D11" t="n">
         <v>2764</v>
@@ -5426,7 +5500,7 @@
         <v>11882</v>
       </c>
       <c r="F11" t="n">
-        <v>8.699999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="G11" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
docs(meta-learning): update content metrics spreadsheet
- Topic Detail: meta-learning row added (5192 words, 11 sections,
  14 TheoremBlocks, 61 display eqs, 455 inline-math, 40 refs all
  with URLs).
- Domain Summary: bayesian-ml row recomputed (now 8 topics, avg 8283
  words, avg 9.4 sections, 1 below 3k threshold, 0 below 7-section
  threshold, 0 missing refs).
- Gap Analysis: no new entries — meta-learning is above all gap
  thresholds.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/formalml-content-metrics.xlsx
+++ b/docs/formalml-content-metrics.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R62"/>
+  <dimension ref="A1:R63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5039,6 +5039,80 @@
       <c r="R62" t="inlineStr">
         <is>
           <t>Motivation: when linear partitions fail, The KDE substrate and the mode-finding picture, Mean-shift as gradient ascent on f_h, Convergence theory, Bandwidth resolution and the mode tree, Kernel-function choice, From trajectories to clusters, Practical mean-shift, k-means as the h-to-0 Voronoi limit, GMM-via-EM and soft assignment, Pointers: spectral and density-based clustering, Connections limits and forward pointers</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>bayesian-ml</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Meta-Learning</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>advanced</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>5192</v>
+      </c>
+      <c r="E63" t="n">
+        <v>11</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K63" t="n">
+        <v>4</v>
+      </c>
+      <c r="L63" t="n">
+        <v>14</v>
+      </c>
+      <c r="M63" t="n">
+        <v>61</v>
+      </c>
+      <c r="N63" t="n">
+        <v>455</v>
+      </c>
+      <c r="O63" t="n">
+        <v>40</v>
+      </c>
+      <c r="P63" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>0</v>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Motivation and the task-distribution structure, Gradient-based meta-learning: MAML, First-order approximations and implicit gradients, Bayesian meta-learning: Neural Processes, Metric-learning meta-learning: Prototypical Networks, The hierarchical-Bayes unifying view, PAC-Bayes generalization theory for meta-learning, Convergence guarantees for MAML, Comparative benchmarks and ablations, Computational notes, Connections and limits</t>
         </is>
       </c>
     </row>
@@ -5488,10 +5562,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C11" t="n">
-        <v>8724</v>
+        <v>8283</v>
       </c>
       <c r="D11" t="n">
         <v>2764</v>
@@ -5500,7 +5574,7 @@
         <v>11882</v>
       </c>
       <c r="F11" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="G11" t="n">
         <v>1</v>

</xml_diff>